<commit_message>
Sync: xlsx edits, regenerated page copy, Facebook join link, overrides cleared
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/page-copy/03-创始人故事.xlsx
+++ b/docs/page-copy/03-创始人故事.xlsx
@@ -529,7 +529,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D6" t="str">
-        <v>I, John LONG WOO, and my two sons Caros Woo and Sam, the three of us, have too many legendary stories with the spiritual realm. These experiences make us the first door opener in the spiritual realm and the first explorer of the truth of **spirit (soul)** life.</v>
+        <v xml:space="preserve">I, John LONG WOO, and my two sons Caros Woo and Sam, the three of us, have too many legendary stories with the spiritual realm. These experiences make us the first door opener in the spiritual realm and the first explorer of the truth of **spirit** </v>
       </c>
       <c r="E6" t="str">
         <v>我， John LONG WOO, 和我的两个儿子Caros Woo和Sam，我们父子三人，与灵魂世界有太多传奇的故事。这些经历造就我们是灵魂世界首位开门者，并且是灵魂生命真相的首位探索者。</v>
@@ -598,7 +598,7 @@
         <v>paragraph / other</v>
       </c>
       <c r="D9" t="str">
-        <v>A living person is composed of both the physical body and the **spirit** (the living **spirit**). After death, that **spirit** becomes **spirit (ghost)**. For the billions of **spirits (ghosts)**, the only means of survival is to obtain energy by attaching to human beings. Attachment by **spirits (ghosts)** causes many diseases, such as epilepsy, depression, schizophrenia, and somatic symptom disorders. With the help of master spirits, these conditions can be rapidly improved. For this we created **Woos Spirit Medicine**.</v>
+        <v>A living person is composed of both the physical body and the **spirit (soul)**. After death, that **spirit(soul) ** becomes **spirit (ghost)**. For the billions of **spirits (ghosts)**, the only means of survival is to obtain energy by attaching to human beings. Attachment by **spirits (ghosts)** causes many diseases, such as epilepsy, depression, schizophrenia, and somatic symptom disorders. With the help of master spirits, these conditions can be rapidly improved. For this we created **Woos Spirit Medicine**.</v>
       </c>
       <c r="E9" t="str">
         <v>人活着时是由肉体和灵体组成的，死后灵体成为了鬼魂（spirit ghost），但是数以几十亿的鬼魂生存的唯一手段是通过附体人类获得能量。鬼魂附体导致了很多疾病，例如：癫痫、抑郁、精分、躯体化障碍。在高级控制灵的帮助下，这些病症可以迅速被改善。为此我们创建了**吴氏灵魂医学**。</v>

</xml_diff>